<commit_message>
Cosas vistas el 08-05, correciones a TP2, lista
</commit_message>
<xml_diff>
--- a/Trabajos Prácticos/TP2/graficos.xlsx
+++ b/Trabajos Prácticos/TP2/graficos.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wheatley\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Facultad\Programación Avanzada\Trabajos Prácticos\TP2\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -74,11 +74,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -218,10 +219,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>17</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>23</c:v>
+                  <c:v>208</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -519,10 +520,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>23</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>18</c:v>
+                  <c:v>173</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2112,7 +2113,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" customWidth="1"/>
@@ -2133,7 +2134,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>17</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2141,7 +2142,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>23</v>
+        <v>208</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -2157,7 +2158,7 @@
         <v>2</v>
       </c>
       <c r="B20">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -2165,11 +2166,15 @@
         <v>3</v>
       </c>
       <c r="B21">
-        <v>18</v>
+        <v>173</v>
       </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B26" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>